<commit_message>
Do not make a nullable member's column required for the required keyword alone
</commit_message>
<xml_diff>
--- a/src/Excelsior.Tests/NullableTests.NullDisplay.verified.xlsx
+++ b/src/Excelsior.Tests/NullableTests.NullDisplay.verified.xlsx
@@ -54,15 +54,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <dxfs count="1">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
 </styleSheet>
 </file>
 
@@ -195,53 +186,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:F4"/>
-  <conditionalFormatting sqref="A2:A4">
-    <cfRule type="containsBlanks" dxfId="0" priority="1">
-      <formula>LEN(TRIM(A2))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B4">
-    <cfRule type="containsBlanks" dxfId="0" priority="2">
-      <formula>LEN(TRIM(B2))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C4">
-    <cfRule type="containsBlanks" dxfId="0" priority="3">
-      <formula>LEN(TRIM(C2))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D4">
-    <cfRule type="containsBlanks" dxfId="0" priority="4">
-      <formula>LEN(TRIM(D2))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E4">
-    <cfRule type="containsBlanks" dxfId="0" priority="5">
-      <formula>LEN(TRIM(E2))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F4">
-    <cfRule type="containsBlanks" dxfId="0" priority="6">
-      <formula>LEN(TRIM(F2))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="6">
-    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="This field is required." prompt="Required field" sqref="A2:A4">
-      <formula1>LEN(TRIM(A2))&gt;0</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="This field is required." prompt="Required field" sqref="B2:B4">
-      <formula1>LEN(TRIM(B2))&gt;0</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="This field is required." prompt="Required field" sqref="C2:C4">
-      <formula1>LEN(TRIM(C2))&gt;0</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="This field is required." prompt="Required field" sqref="D2:D4">
-      <formula1>LEN(TRIM(D2))&gt;0</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be one of: Value." prompt="Select one of: Value" sqref="E2:E4">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be one of: Value." prompt="Select one of: Value" sqref="E2:E4">
       <formula1>"Value"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be one of: TRUE, FALSE." prompt="Select one of: TRUE, FALSE" sqref="F2:F4">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be one of: TRUE, FALSE." prompt="Select one of: TRUE, FALSE" sqref="F2:F4">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Do not make a nullable member's column required for the required keyword alone (#282)
</commit_message>
<xml_diff>
--- a/src/Excelsior.Tests/NullableTests.NullDisplay.verified.xlsx
+++ b/src/Excelsior.Tests/NullableTests.NullDisplay.verified.xlsx
@@ -54,15 +54,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <dxfs count="1">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
 </styleSheet>
 </file>
 
@@ -191,55 +182,22 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:F4"/>
-  <conditionalFormatting sqref="A2:A4">
-    <cfRule type="containsBlanks" dxfId="0" priority="1">
-      <formula>LEN(TRIM(A2))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B4">
-    <cfRule type="containsBlanks" dxfId="0" priority="2">
-      <formula>LEN(TRIM(B2))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C4">
-    <cfRule type="containsBlanks" dxfId="0" priority="3">
-      <formula>LEN(TRIM(C2))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D4">
-    <cfRule type="containsBlanks" dxfId="0" priority="4">
-      <formula>LEN(TRIM(D2))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E4">
-    <cfRule type="containsBlanks" dxfId="0" priority="5">
-      <formula>LEN(TRIM(E2))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F4">
-    <cfRule type="containsBlanks" dxfId="0" priority="6">
-      <formula>LEN(TRIM(F2))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="6">
-    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a number." prompt="Required field" sqref="A2:A4">
+  <dataValidations count="5">
+    <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a number." sqref="A2:A4">
       <formula1>ISNUMBER(A2)</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="This field is required." prompt="Required field" sqref="B2:B4">
-      <formula1>LEN(TRIM(B2))&gt;0</formula1>
-    </dataValidation>
-    <dataValidation type="date" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a valid date and time.&#10;yyyy-MM-dd HH:mm:ss" prompt="Date and time as yyyy-MM-dd HH:mm:ss" sqref="C2:C4">
+    <dataValidation type="date" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a valid date and time.&#10;yyyy-MM-dd HH:mm:ss" prompt="Date and time as yyyy-MM-dd HH:mm:ss" sqref="C2:C4">
       <formula1>2</formula1>
       <formula2>2958465</formula2>
     </dataValidation>
-    <dataValidation type="date" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a valid date.&#10;yyyy-MM-dd" prompt="Date as yyyy-MM-dd" sqref="D2:D4">
+    <dataValidation type="date" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a valid date.&#10;yyyy-MM-dd" prompt="Date as yyyy-MM-dd" sqref="D2:D4">
       <formula1>2</formula1>
       <formula2>2958465</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be one of: Value." prompt="Select one of: Value" sqref="E2:E4">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be one of: Value." prompt="Select one of: Value" sqref="E2:E4">
       <formula1>"Value"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be one of: TRUE, FALSE." prompt="Select one of: TRUE, FALSE" sqref="F2:F4">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be one of: TRUE, FALSE." prompt="Select one of: TRUE, FALSE" sqref="F2:F4">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>